<commit_message>
Widen SO textarea (width:100%), update sample XLSX+HTML (Option 1/2, no num prefix, SO defaults)
</commit_message>
<xml_diff>
--- a/sample_output_v3.xlsx
+++ b/sample_output_v3.xlsx
@@ -106,6 +106,12 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="00374151"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="001E3A8A"/>
       <sz val="9"/>
     </font>
@@ -136,12 +142,6 @@
       <name val="Calibri"/>
       <color rgb="001E3A8A"/>
       <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00374151"/>
-      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -348,7 +348,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -422,32 +422,39 @@
     <xf numFmtId="0" fontId="13" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -474,7 +481,6 @@
     <xf numFmtId="3" fontId="25" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="21" fillId="2" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -843,7 +849,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1168,7 +1174,7 @@
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">    📅 Timeline &amp; แผนการดำเนินงาน</t>
+          <t xml:space="preserve">    🎁 Special Offers</t>
         </is>
       </c>
     </row>
@@ -1180,236 +1186,308 @@
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>ผู้รับผิดชอบ</t>
+          <t>รายการ</t>
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>Task / กระบวนการ</t>
-        </is>
-      </c>
-      <c r="D19" s="11" t="inlineStr">
-        <is>
           <t>รายละเอียด</t>
         </is>
       </c>
-      <c r="E19" s="11" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="F19" s="11" t="inlineStr">
-        <is>
-          <t>วันที่เริ่ม</t>
-        </is>
-      </c>
-      <c r="G19" s="11" t="inlineStr">
-        <is>
-          <t>วันที่สิ้นสุด</t>
-        </is>
-      </c>
-      <c r="H19" s="11" t="inlineStr"/>
-      <c r="I19" s="11" t="inlineStr"/>
-    </row>
-    <row r="20" ht="40" customHeight="1">
+      <c r="D19" s="27" t="n"/>
+      <c r="E19" s="27" t="n"/>
+      <c r="F19" s="27" t="n"/>
+      <c r="G19" s="27" t="n"/>
+      <c r="H19" s="27" t="n"/>
+      <c r="I19" s="12" t="n"/>
+    </row>
+    <row r="20" ht="44" customHeight="1">
       <c r="A20" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="B20" s="27" t="inlineStr">
+      <c r="B20" s="28" t="inlineStr">
+        <is>
+          <t>ข้อเสนอพิเศษ</t>
+        </is>
+      </c>
+      <c r="C20" s="14" t="inlineStr">
+        <is>
+          <t>สำหรับการสมัครใช้งานแพ็กเกจ (สัญญา 1 ปี) — 10 ฟรี 2 เมื่อชำระภายในเดือน</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="44" customHeight="1">
+      <c r="A21" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="B21" s="29" t="inlineStr">
+        <is>
+          <t>บริการ</t>
+        </is>
+      </c>
+      <c r="C21" s="20" t="inlineStr">
+        <is>
+          <t>• ไม่มีค่า MA  • ขึ้นระบบให้ฟรี  • ไม่มีค่าเช่า Cloud
+• Support ทุกวัน 08.30–17.30 น.  • รองรับ Multi Company  • Training ฟรี 3 ครั้ง</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="6" customHeight="1">
+      <c r="A22" s="7" t="n"/>
+      <c r="B22" s="7" t="n"/>
+      <c r="C22" s="7" t="n"/>
+      <c r="D22" s="7" t="n"/>
+      <c r="E22" s="7" t="n"/>
+      <c r="F22" s="7" t="n"/>
+      <c r="G22" s="7" t="n"/>
+      <c r="H22" s="7" t="n"/>
+      <c r="I22" s="7" t="n"/>
+    </row>
+    <row r="23" ht="28" customHeight="1">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    📅 Timeline &amp; แผนการดำเนินงาน</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="28" customHeight="1">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>ผู้รับผิดชอบ</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>Task / กระบวนการ</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>รายละเอียด</t>
+        </is>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>วันที่เริ่ม</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="inlineStr">
+        <is>
+          <t>วันที่สิ้นสุด</t>
+        </is>
+      </c>
+      <c r="H24" s="11" t="inlineStr"/>
+      <c r="I24" s="11" t="inlineStr"/>
+    </row>
+    <row r="25" ht="40" customHeight="1">
+      <c r="A25" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="B25" s="30" t="inlineStr">
         <is>
           <t>HumanSoft</t>
         </is>
       </c>
-      <c r="C20" s="28" t="inlineStr">
+      <c r="C25" s="31" t="inlineStr">
         <is>
           <t>Demo &amp; Requirement
 Gathering</t>
         </is>
       </c>
-      <c r="D20" s="14" t="inlineStr">
+      <c r="D25" s="14" t="inlineStr">
         <is>
           <t>นำเสนอระบบ + เก็บ Req</t>
         </is>
       </c>
-      <c r="E20" s="23" t="inlineStr">
+      <c r="E25" s="23" t="inlineStr">
         <is>
           <t>In progress</t>
         </is>
       </c>
-      <c r="F20" s="29" t="inlineStr">
+      <c r="F25" s="32" t="inlineStr">
         <is>
           <t>2/6/2569</t>
         </is>
       </c>
-      <c r="G20" s="29" t="inlineStr">
+      <c r="G25" s="32" t="inlineStr">
         <is>
           <t>13/6/2569</t>
         </is>
       </c>
-      <c r="H20" s="18" t="inlineStr"/>
-      <c r="I20" s="18" t="inlineStr"/>
-    </row>
-    <row r="21" ht="40" customHeight="1">
-      <c r="A21" s="19" t="n">
+      <c r="H25" s="18" t="inlineStr"/>
+      <c r="I25" s="18" t="inlineStr"/>
+    </row>
+    <row r="26" ht="40" customHeight="1">
+      <c r="A26" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="B21" s="30" t="inlineStr">
+      <c r="B26" s="33" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="C21" s="31" t="inlineStr">
+      <c r="C26" s="34" t="inlineStr">
         <is>
           <t>ตรวจสอบข้อมูลพนักงาน</t>
         </is>
       </c>
-      <c r="D21" s="20" t="inlineStr">
+      <c r="D26" s="20" t="inlineStr">
         <is>
           <t>Export จากระบบเดิม</t>
         </is>
       </c>
-      <c r="E21" s="17" t="inlineStr">
+      <c r="E26" s="17" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="F21" s="32" t="inlineStr">
+      <c r="F26" s="35" t="inlineStr">
         <is>
           <t>9/6/2569</t>
         </is>
       </c>
-      <c r="G21" s="32" t="inlineStr">
+      <c r="G26" s="35" t="inlineStr">
         <is>
           <t>13/6/2569</t>
         </is>
       </c>
-      <c r="H21" s="22" t="inlineStr"/>
-      <c r="I21" s="22" t="inlineStr"/>
-    </row>
-    <row r="22" ht="40" customHeight="1">
-      <c r="A22" s="13" t="n">
+      <c r="H26" s="22" t="inlineStr"/>
+      <c r="I26" s="22" t="inlineStr"/>
+    </row>
+    <row r="27" ht="40" customHeight="1">
+      <c r="A27" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="B22" s="27" t="inlineStr">
+      <c r="B27" s="30" t="inlineStr">
         <is>
           <t>HumanSoft</t>
         </is>
       </c>
-      <c r="C22" s="28" t="inlineStr">
+      <c r="C27" s="31" t="inlineStr">
         <is>
           <t>ติดตั้งและ Setup ระบบ</t>
         </is>
       </c>
-      <c r="D22" s="14" t="inlineStr">
+      <c r="D27" s="14" t="inlineStr">
         <is>
           <t>Config ตาม Req</t>
         </is>
       </c>
-      <c r="E22" s="17" t="inlineStr">
+      <c r="E27" s="17" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="F22" s="29" t="inlineStr">
+      <c r="F27" s="32" t="inlineStr">
         <is>
           <t>1/7/2569</t>
         </is>
       </c>
-      <c r="G22" s="29" t="inlineStr">
+      <c r="G27" s="32" t="inlineStr">
         <is>
           <t>15/7/2569</t>
         </is>
       </c>
-      <c r="H22" s="18" t="inlineStr"/>
-      <c r="I22" s="18" t="inlineStr"/>
-    </row>
-    <row r="23" ht="40" customHeight="1">
-      <c r="A23" s="19" t="n">
+      <c r="H27" s="18" t="inlineStr"/>
+      <c r="I27" s="18" t="inlineStr"/>
+    </row>
+    <row r="28" ht="40" customHeight="1">
+      <c r="A28" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="B23" s="27" t="inlineStr">
+      <c r="B28" s="30" t="inlineStr">
         <is>
           <t>HumanSoft</t>
         </is>
       </c>
-      <c r="C23" s="31" t="inlineStr">
+      <c r="C28" s="34" t="inlineStr">
         <is>
           <t>Training ผู้ดูแลระบบ</t>
         </is>
       </c>
-      <c r="D23" s="20" t="inlineStr">
+      <c r="D28" s="20" t="inlineStr">
         <is>
           <t>อบรม Admin 2 วัน</t>
         </is>
       </c>
-      <c r="E23" s="17" t="inlineStr">
+      <c r="E28" s="17" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="F23" s="32" t="inlineStr">
+      <c r="F28" s="35" t="inlineStr">
         <is>
           <t>14/7/2569</t>
         </is>
       </c>
-      <c r="G23" s="32" t="inlineStr">
+      <c r="G28" s="35" t="inlineStr">
         <is>
           <t>31/7/2569</t>
         </is>
       </c>
-      <c r="H23" s="22" t="inlineStr"/>
-      <c r="I23" s="22" t="inlineStr"/>
-    </row>
-    <row r="24" ht="40" customHeight="1">
-      <c r="A24" s="13" t="n">
+      <c r="H28" s="22" t="inlineStr"/>
+      <c r="I28" s="22" t="inlineStr"/>
+    </row>
+    <row r="29" ht="40" customHeight="1">
+      <c r="A29" s="13" t="n">
         <v>5</v>
       </c>
-      <c r="B24" s="33" t="inlineStr">
+      <c r="B29" s="36" t="inlineStr">
         <is>
           <t>Humansoft / Client</t>
         </is>
       </c>
-      <c r="C24" s="28" t="inlineStr">
+      <c r="C29" s="31" t="inlineStr">
         <is>
           <t>🚀 Go Live</t>
         </is>
       </c>
-      <c r="D24" s="14" t="inlineStr">
+      <c r="D29" s="14" t="inlineStr">
         <is>
           <t>เปิดใช้งานจริง</t>
         </is>
       </c>
-      <c r="E24" s="17" t="inlineStr">
+      <c r="E29" s="17" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="F24" s="29" t="inlineStr">
+      <c r="F29" s="32" t="inlineStr">
         <is>
           <t>15/8/2569</t>
         </is>
       </c>
-      <c r="G24" s="29" t="inlineStr">
+      <c r="G29" s="32" t="inlineStr">
         <is>
           <t>15/8/2569</t>
         </is>
       </c>
-      <c r="H24" s="18" t="inlineStr"/>
-      <c r="I24" s="18" t="inlineStr"/>
-    </row>
-    <row r="25" ht="5" customHeight="1">
-      <c r="A25" s="34" t="n"/>
-      <c r="B25" s="34" t="n"/>
-      <c r="C25" s="34" t="n"/>
-      <c r="D25" s="34" t="n"/>
-      <c r="E25" s="34" t="n"/>
-      <c r="F25" s="34" t="n"/>
-      <c r="G25" s="34" t="n"/>
-      <c r="H25" s="34" t="n"/>
-      <c r="I25" s="34" t="n"/>
+      <c r="H29" s="18" t="inlineStr"/>
+      <c r="I29" s="18" t="inlineStr"/>
+    </row>
+    <row r="30" ht="5" customHeight="1">
+      <c r="A30" s="37" t="n"/>
+      <c r="B30" s="37" t="n"/>
+      <c r="C30" s="37" t="n"/>
+      <c r="D30" s="37" t="n"/>
+      <c r="E30" s="37" t="n"/>
+      <c r="F30" s="37" t="n"/>
+      <c r="G30" s="37" t="n"/>
+      <c r="H30" s="37" t="n"/>
+      <c r="I30" s="37" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="25">
+  <mergeCells count="29">
     <mergeCell ref="E12:F12"/>
     <mergeCell ref="G12:H12"/>
     <mergeCell ref="C8:I8"/>
@@ -1418,7 +1496,9 @@
     <mergeCell ref="C7:I7"/>
     <mergeCell ref="E14:F14"/>
     <mergeCell ref="A6:B6"/>
+    <mergeCell ref="C19:I19"/>
     <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A23:I23"/>
     <mergeCell ref="C6:I6"/>
     <mergeCell ref="E13:F13"/>
     <mergeCell ref="G13:H13"/>
@@ -1430,10 +1510,12 @@
     <mergeCell ref="G15:H15"/>
     <mergeCell ref="E11:F11"/>
     <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C20:I20"/>
     <mergeCell ref="G14:H14"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="E16:F16"/>
     <mergeCell ref="G16:H16"/>
+    <mergeCell ref="C21:I21"/>
     <mergeCell ref="A2:G2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1487,9 +1569,9 @@
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Professional vs Standard  |  51–75 คน  |  ราย 1 ปี</t>
+      <c r="A3" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  แพ็กเกจแนะนำสำหรับพนักงาน 51–75 คน</t>
         </is>
       </c>
     </row>
@@ -1504,19 +1586,19 @@
       <c r="H4" s="7" t="n"/>
     </row>
     <row r="5" ht="34" customHeight="1">
-      <c r="A5" s="36" t="inlineStr">
+      <c r="A5" s="39" t="inlineStr">
         <is>
           <t>รายการ</t>
         </is>
       </c>
-      <c r="C5" s="37" t="inlineStr">
-        <is>
-          <t>🅐 ตัวเลือก A — Professional</t>
-        </is>
-      </c>
-      <c r="F5" s="38" t="inlineStr">
-        <is>
-          <t>🅑 ตัวเลือก B — Standard</t>
+      <c r="C5" s="40" t="inlineStr">
+        <is>
+          <t>Option 1 — Professional</t>
+        </is>
+      </c>
+      <c r="F5" s="41" t="inlineStr">
+        <is>
+          <t>Option 2 — Standard</t>
         </is>
       </c>
     </row>
@@ -1526,12 +1608,12 @@
           <t>แพ็กเกจ</t>
         </is>
       </c>
-      <c r="C6" s="39" t="inlineStr">
+      <c r="C6" s="42" t="inlineStr">
         <is>
           <t>Professional</t>
         </is>
       </c>
-      <c r="F6" s="40" t="inlineStr">
+      <c r="F6" s="43" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
@@ -1543,12 +1625,12 @@
           <t>จำนวนพนักงาน</t>
         </is>
       </c>
-      <c r="C7" s="39" t="inlineStr">
+      <c r="C7" s="42" t="inlineStr">
         <is>
           <t>51–75 คน</t>
         </is>
       </c>
-      <c r="F7" s="40" t="inlineStr">
+      <c r="F7" s="43" t="inlineStr">
         <is>
           <t>51–75 คน</t>
         </is>
@@ -1560,12 +1642,12 @@
           <t>ระยะเวลา</t>
         </is>
       </c>
-      <c r="C8" s="39" t="inlineStr">
+      <c r="C8" s="42" t="inlineStr">
         <is>
           <t>ราย 1 ปี</t>
         </is>
       </c>
-      <c r="F8" s="40" t="inlineStr">
+      <c r="F8" s="43" t="inlineStr">
         <is>
           <t>ราย 1 ปี</t>
         </is>
@@ -1577,12 +1659,12 @@
           <t>โปรโมชั่น</t>
         </is>
       </c>
-      <c r="C9" s="39" t="inlineStr">
+      <c r="C9" s="42" t="inlineStr">
         <is>
           <t>ฟรี 3 เดือน</t>
         </is>
       </c>
-      <c r="F9" s="40" t="inlineStr">
+      <c r="F9" s="43" t="inlineStr">
         <is>
           <t>ฟรี 2 เดือน</t>
         </is>
@@ -1594,10 +1676,10 @@
           <t>ราคาปกติ (ไม่มีโปร)</t>
         </is>
       </c>
-      <c r="C10" s="41" t="n">
+      <c r="C10" s="44" t="n">
         <v>98670</v>
       </c>
-      <c r="F10" s="42" t="n">
+      <c r="F10" s="45" t="n">
         <v>40680</v>
       </c>
     </row>
@@ -1607,27 +1689,27 @@
           <t>ส่วนลดพิเศษ 5%</t>
         </is>
       </c>
-      <c r="C11" s="39" t="inlineStr">
+      <c r="C11" s="42" t="inlineStr">
         <is>
           <t>−3,795 บาท</t>
         </is>
       </c>
-      <c r="F11" s="40" t="inlineStr">
+      <c r="F11" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="12" ht="38" customHeight="1">
-      <c r="A12" s="43" t="inlineStr">
+      <c r="A12" s="46" t="inlineStr">
         <is>
           <t>💎 ยอดสุทธิ</t>
         </is>
       </c>
-      <c r="C12" s="44" t="n">
+      <c r="C12" s="47" t="n">
         <v>72105</v>
       </c>
-      <c r="F12" s="44" t="n">
+      <c r="F12" s="47" t="n">
         <v>33900</v>
       </c>
     </row>
@@ -1637,10 +1719,10 @@
           <t>อัตราเดือนละ</t>
         </is>
       </c>
-      <c r="C13" s="41" t="n">
+      <c r="C13" s="44" t="n">
         <v>7590</v>
       </c>
-      <c r="F13" s="42" t="n">
+      <c r="F13" s="45" t="n">
         <v>3390</v>
       </c>
     </row>
@@ -1650,26 +1732,26 @@
           <t>💚 ประหยัดรวม</t>
         </is>
       </c>
-      <c r="C14" s="39" t="inlineStr">
+      <c r="C14" s="42" t="inlineStr">
         <is>
           <t>26,565 บาท (27%)</t>
         </is>
       </c>
-      <c r="F14" s="40" t="inlineStr">
+      <c r="F14" s="43" t="inlineStr">
         <is>
           <t>6,780 บาท (17%)</t>
         </is>
       </c>
     </row>
     <row r="15" ht="5" customHeight="1">
-      <c r="A15" s="34" t="n"/>
-      <c r="B15" s="34" t="n"/>
-      <c r="C15" s="34" t="n"/>
-      <c r="D15" s="34" t="n"/>
-      <c r="E15" s="34" t="n"/>
-      <c r="F15" s="34" t="n"/>
-      <c r="G15" s="34" t="n"/>
-      <c r="H15" s="34" t="n"/>
+      <c r="A15" s="37" t="n"/>
+      <c r="B15" s="37" t="n"/>
+      <c r="C15" s="37" t="n"/>
+      <c r="D15" s="37" t="n"/>
+      <c r="E15" s="37" t="n"/>
+      <c r="F15" s="37" t="n"/>
+      <c r="G15" s="37" t="n"/>
+      <c r="H15" s="37" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="32">
@@ -1751,7 +1833,7 @@
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="35" t="inlineStr">
+      <c r="A3" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  ✓ = ต้องการใช้งาน</t>
         </is>
@@ -1776,13 +1858,13 @@
           <t>ฟีเจอร์ที่เลือก</t>
         </is>
       </c>
-      <c r="D5" s="45" t="n"/>
+      <c r="D5" s="27" t="n"/>
       <c r="E5" s="12" t="n"/>
     </row>
     <row r="6" ht="26" customHeight="1">
-      <c r="A6" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  1. Channel</t>
+      <c r="A6" s="48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Channel</t>
         </is>
       </c>
     </row>
@@ -1813,9 +1895,9 @@
       </c>
     </row>
     <row r="9" ht="26" customHeight="1">
-      <c r="A9" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  7. ลงเวลาการทำงาน</t>
+      <c r="A9" s="48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ลงเวลาการทำงาน</t>
         </is>
       </c>
     </row>
@@ -1859,9 +1941,9 @@
       </c>
     </row>
     <row r="13" ht="26" customHeight="1">
-      <c r="A13" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  8. เอกสารและการอนุมัติ</t>
+      <c r="A13" s="48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  เอกสารและการอนุมัติ</t>
         </is>
       </c>
     </row>
@@ -1905,9 +1987,9 @@
       </c>
     </row>
     <row r="17" ht="26" customHeight="1">
-      <c r="A17" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  9. การคำนวณเงินเดือน</t>
+      <c r="A17" s="48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  การคำนวณเงินเดือน</t>
         </is>
       </c>
     </row>
@@ -1951,9 +2033,9 @@
       </c>
     </row>
     <row r="21" ht="26" customHeight="1">
-      <c r="A21" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  10. รายงาน</t>
+      <c r="A21" s="48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  รายงาน</t>
         </is>
       </c>
     </row>
@@ -1971,9 +2053,9 @@
       </c>
     </row>
     <row r="23" ht="26" customHeight="1">
-      <c r="A23" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  11. HRD</t>
+      <c r="A23" s="48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  การเรียนรู้และพัฒนาองค์กร (HRD)</t>
         </is>
       </c>
     </row>
@@ -2004,9 +2086,9 @@
       </c>
     </row>
     <row r="26" ht="26" customHeight="1">
-      <c r="A26" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  5. ระบบความปลอดภัย</t>
+      <c r="A26" s="48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ระบบความปลอดภัย</t>
         </is>
       </c>
     </row>
@@ -2037,11 +2119,11 @@
       </c>
     </row>
     <row r="29" ht="5" customHeight="1">
-      <c r="A29" s="34" t="n"/>
-      <c r="B29" s="34" t="n"/>
-      <c r="C29" s="34" t="n"/>
-      <c r="D29" s="34" t="n"/>
-      <c r="E29" s="34" t="n"/>
+      <c r="A29" s="37" t="n"/>
+      <c r="B29" s="37" t="n"/>
+      <c r="C29" s="37" t="n"/>
+      <c r="D29" s="37" t="n"/>
+      <c r="E29" s="37" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="26">

</xml_diff>